<commit_message>
Add Dalhousie/SDUFE Instructor of Economics under Shandong and track three referees.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/application/recommendation_letters_to_send.xlsx
+++ b/application/recommendation_letters_to_send.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -604,6 +604,43 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Dalhousie University (joint with SDUFE, Jinan; F825P)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Instructor of Economics</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>PeopleAdmin</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://dal.peopleadmin.ca/postings/22333</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Three referees (list of contacts; letters if requested)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>To send</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Duke Kunshan University application materials and update trackers
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/application/recommendation_letters_to_send.xlsx
+++ b/application/recommendation_letters_to_send.xlsx
@@ -494,111 +494,111 @@
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Fudan University</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Assistant Professor</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>2026-11-01</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>econsearch@fudan.edu.cn</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Recommendation letter</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>To send</t>
         </is>
       </c>
     </row>
     <row r="3" ht="36" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Chung-Hua Institution for Economic Research (CIER)</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Assistant Research Fellow</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Email (writers send letters directly)</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>fangru@cier.edu.tw</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Three recommendation letters</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CUHK-SZ (Zhang Yiming Project, PR2026/049/01)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Post Doctoral Fellow</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>zhangyiming@cuhk.edu.cn</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Two recommendation letters</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>To send</t>
         </is>
       </c>
     </row>
     <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>CUHK-SZ (Zhang Yiming Project, PR2026/049/01)</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Post Doctoral Fellow</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>zhangyiming@cuhk.edu.cn</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Two recommendation letters</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Dalhousie University (joint with SDUFE, Jinan; F825P)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Instructor of Economics</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>PeopleAdmin</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://dal.peopleadmin.ca/postings/22333</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Three referees (list of contacts; letters if requested)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>To send</t>
         </is>
@@ -607,32 +607,32 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Dalhousie University (joint with SDUFE, Jinan; F825P)</t>
+          <t>Chung-Hua Institution for Economic Research (CIER)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Instructor of Economics</t>
+          <t>Assistant Research Fellow</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-11-20</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>PeopleAdmin</t>
+          <t>Email (writers send letters directly)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://dal.peopleadmin.ca/postings/22333</t>
+          <t>fangru@cier.edu.tw</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Three referees (list of contacts; letters if requested)</t>
+          <t>Three recommendation letters</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">

</xml_diff>

<commit_message>
Add Fudan application materials and update trackers
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/application/recommendation_letters_to_send.xlsx
+++ b/application/recommendation_letters_to_send.xlsx
@@ -496,7 +496,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Fudan University</t>
+          <t>Fudan University (School of Economics)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -511,7 +511,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Email (writers send letters directly)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,7 +521,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Recommendation letter</t>
+          <t>Three recommendation letters</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -600,7 +600,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>To send</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -637,7 +637,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>To send</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Referees and Sent? columns to recommendation letters tracker
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/application/recommendation_letters_to_send.xlsx
+++ b/application/recommendation_letters_to_send.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -457,39 +457,49 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Position</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Deadline</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>How to apply</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Email / contact</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Materials</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Referees</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
         <is>
           <t>Status</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Sent?</t>
         </is>
       </c>
     </row>
@@ -526,7 +536,17 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>Pak Hung Au, Kohei Kawaguchi, Kei Kawai</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>To send</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -563,7 +583,17 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>Kohei Kawaguchi, Kei Kawai</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>To send</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -600,7 +630,17 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
+          <t>Pak Hung Au, Kohei Kawaguchi, Kei Kawai</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>Pending</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -637,7 +677,17 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
+          <t>Pak Hung Au, Kohei Kawaguchi, Kei Kawai</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>Pending</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Style recommendation letters tracker header and status colors
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/application/recommendation_letters_to_send.xlsx
+++ b/application/recommendation_letters_to_send.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recommendation letters" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Recommendation letters'!$A$1:$G$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Recommendation letters'!$A$5:$I$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,11 +28,39 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="005B6B7A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00333333"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -41,7 +69,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002F5496"/>
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -55,29 +93,51 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="00D9D9D9"/>
       </left>
       <right style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="00D9D9D9"/>
       </right>
       <top style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="00D9D9D9"/>
       </top>
       <bottom style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="00D9D9D9"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -444,255 +504,283 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Recommendation Letters to Send Out</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Ke Cheng Hsu (Clio) · Department of Economics, HKUST · Updated 29 October 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Only send rows with Status "To send". Leave "Pending" rows unsent. After sending, change Sent? from No to Yes. Use the Referees column to choose which letters to attach. Rows ordered by deadline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Position</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Deadline</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>How to apply</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Email / contact</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Materials</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Referees</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Sent?</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="36" customHeight="1">
-      <c r="A2" t="inlineStr">
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Fudan University (School of Economics)</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Assistant Professor</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>2026-11-01</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Email (writers send letters directly)</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>econsearch@fudan.edu.cn</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>Three recommendation letters</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>Pak Hung Au, Kohei Kawaguchi, Kei Kawai</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>To send</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I6" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="36" customHeight="1">
-      <c r="A3" t="inlineStr">
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>CUHK-SZ (Zhang Yiming Project, PR2026/049/01)</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Post Doctoral Fellow</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>2026-11-01</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>zhangyiming@cuhk.edu.cn</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>Two recommendation letters</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Kohei Kawaguchi, Kei Kawai</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>To send</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I7" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1">
-      <c r="A4" t="inlineStr">
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Dalhousie University (joint with SDUFE, Jinan; F825P)</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Instructor of Economics</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>PeopleAdmin</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>https://dal.peopleadmin.ca/postings/22333</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>Three referees (list of contacts; letters if requested)</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G8" s="8" t="inlineStr">
         <is>
           <t>Pak Hung Au, Kohei Kawaguchi, Kei Kawai</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H8" s="9" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I8" s="10" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Chung-Hua Institution for Economic Research (CIER)</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Assistant Research Fellow</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>2026-12-31</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>Email (writers send letters directly)</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>fangru@cier.edu.tw</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>Three recommendation letters</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G9" s="8" t="inlineStr">
         <is>
           <t>Pak Hung Au, Kohei Kawaguchi, Kei Kawai</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H9" s="9" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I9" s="10" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G4"/>
+  <autoFilter ref="A5:I9"/>
+  <mergeCells count="3">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A2:I2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add JOE faculty openings and update application trackers
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/application/recommendation_letters_to_send.xlsx
+++ b/application/recommendation_letters_to_send.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recommendation letters" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Recommendation letters'!$A$5:$I$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Recommendation letters'!$A$5:$I$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -504,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -730,52 +730,381 @@
     <row r="9" ht="36" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
+          <t>CUEB ISEM (Capital University of Economics and Business)</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Asst/Assoc/Full Professor</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Email (writers send letters)</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>hr_isem@163.com</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Two recommendation letters</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Kohei Kawaguchi, Kei Kawai</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>HUST School of Economics</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Asst/Assoc/Full Professor</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>JOE or email (writers)</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>eco_hust@163.com</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Three recommendation letters</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Pak Hung Au, Kohei Kawaguchi, Kei Kawai</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>IEAS Academia Sinica</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Asst/Assoc/Research Fellow</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>JOE / writers send letters</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>searchcommit@econ.sinica.edu.tw</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Three recommendation letters</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Pak Hung Au, Kohei Kawaguchi, Kei Kawai</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Jinan University IESR (tenure-track)</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Asst/Assoc/Full Professor</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Writers send letters</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>iesr_job@126.com</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Three recommendation letters</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Pak Hung Au, Kohei Kawaguchi, Kei Kawai</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I12" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>DUFE IAER (Dongbei University of Finance and Economics)</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Asst/Assoc/Full Professor</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>2026-12-15</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>JOE (writers upload letters)</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111478252</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Three recommendation letters</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Pak Hung Au, Kohei Kawaguchi, Kei Kawai</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Hunan University SET</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Asst/Assoc/Full Professor</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>JOE (writers upload letters)</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111478275</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Three recommendation letters</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Pak Hung Au, Kohei Kawaguchi, Kei Kawai</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I14" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
           <t>Chung-Hua Institution for Economic Research (CIER)</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Assistant Research Fellow</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>2026-12-31</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>Email (writers send letters directly)</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>fangru@cier.edu.tw</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>Three recommendation letters</t>
         </is>
       </c>
-      <c r="G9" s="8" t="inlineStr">
+      <c r="G15" s="8" t="inlineStr">
         <is>
           <t>Pak Hung Au, Kohei Kawaguchi, Kei Kawai</t>
         </is>
       </c>
-      <c r="H9" s="9" t="inlineStr">
+      <c r="H15" s="9" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="I9" s="10" t="inlineStr">
+      <c r="I15" s="10" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Jinan University IESR</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>International Research Fellow</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>2027-07-31</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>JOE or email (writers)</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>iesr_job@126.com</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Letters of reference</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Pak Hung Au, Kohei Kawaguchi, Kei Kawai</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I16" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:I9"/>
+  <autoFilter ref="A5:I16"/>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A3:I3"/>

</xml_diff>

<commit_message>
Add NCU Economics and Industrial Economics JOE openings
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/application/recommendation_letters_to_send.xlsx
+++ b/application/recommendation_letters_to_send.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recommendation letters" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Recommendation letters'!$A$5:$I$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Recommendation letters'!$A$5:$I$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -504,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -918,17 +918,17 @@
     <row r="13" ht="36" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>DUFE IAER (Dongbei University of Finance and Economics)</t>
+          <t>NCU Economics (National Central University)</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Asst/Assoc/Full Professor</t>
+          <t>Asst Professor or above</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>2026-12-15</t>
+          <t>2026-12-02</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111478252</t>
+          <t>ncu66301@ncu.edu.tw</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -965,7 +965,7 @@
     <row r="14" ht="36" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>Hunan University SET</t>
+          <t>NCU Industrial Economics</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
@@ -975,17 +975,17 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>2026-12-31</t>
+          <t>2026-12-12</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>JOE (writers upload letters)</t>
+          <t>Email (writers send letters)</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111478275</t>
+          <t>ncu6450@ncu.edu.tw</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
@@ -1012,27 +1012,27 @@
     <row r="15" ht="36" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>Chung-Hua Institution for Economic Research (CIER)</t>
+          <t>DUFE IAER (Dongbei University of Finance and Economics)</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Assistant Research Fellow</t>
+          <t>Asst/Assoc/Full Professor</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>2026-12-31</t>
+          <t>2026-12-15</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Email (writers send letters directly)</t>
+          <t>JOE (writers upload letters)</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>fangru@cier.edu.tw</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111478252</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -1059,52 +1059,146 @@
     <row r="16" ht="36" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
+          <t>Hunan University SET</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Asst/Assoc/Full Professor</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>JOE (writers upload letters)</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111478275</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Three recommendation letters</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Pak Hung Au, Kohei Kawaguchi, Kei Kawai</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I16" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="36" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Chung-Hua Institution for Economic Research (CIER)</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Assistant Research Fellow</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Email (writers send letters directly)</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>fangru@cier.edu.tw</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Three recommendation letters</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Pak Hung Au, Kohei Kawaguchi, Kei Kawai</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I17" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="36" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
           <t>Jinan University IESR</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>International Research Fellow</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>2027-07-31</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>JOE or email (writers)</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="E18" s="8" t="inlineStr">
         <is>
           <t>iesr_job@126.com</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr">
+      <c r="F18" s="8" t="inlineStr">
         <is>
           <t>Letters of reference</t>
         </is>
       </c>
-      <c r="G16" s="8" t="inlineStr">
+      <c r="G18" s="8" t="inlineStr">
         <is>
           <t>Pak Hung Au, Kohei Kawaguchi, Kei Kawai</t>
         </is>
       </c>
-      <c r="H16" s="9" t="inlineStr">
+      <c r="H18" s="9" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="I16" s="10" t="inlineStr">
+      <c r="I18" s="10" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:I16"/>
+  <autoFilter ref="A5:I18"/>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A3:I3"/>

</xml_diff>